<commit_message>
trennung von predict und create_excel
</commit_message>
<xml_diff>
--- a/data/predictions.xlsx
+++ b/data/predictions.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,151 +447,226 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-11 19:30:00</t>
+          <t>2026-03-12 19:00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cleveland Cavaliers</t>
+          <t>Philadelphia 76ers</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Orlando Magic</t>
+          <t>Detroit Pistons</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5571080187350942</v>
+        <v>0.6845906696876617</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-11 20:00:00</t>
+          <t>2026-03-12 19:00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Indiana Pacers</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>New Orleans Pelicans</t>
+          <t>Phoenix Suns</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.5142161141394647</v>
+        <v>0.338383779640849</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-11 21:00:00</t>
+          <t>2026-03-12 19:00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Utah Jazz</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Washington Wizards</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.3859660484608027</v>
+        <v>0.8041494742951564</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-11 22:00:00</t>
+          <t>2026-03-12 19:30:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Denver Nuggets</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Brooklyn Nets</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Denver Nuggets</t>
+          <t>Atlanta Hawks</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.5896213374417394</v>
+        <v>0.8979168904111741</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-11 22:00:00</t>
+          <t>2026-03-12 19:30:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sacramento Kings</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Milwaukee Bucks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Charlotte Hornets</t>
+          <t>Miami Heat</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.417710854441212</v>
+        <v>0.7569148209082387</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-11 22:30:00</t>
+          <t>2026-03-12 20:00:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>Dallas Mavericks</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LA Clippers</t>
+          <t>Memphis Grizzlies</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.6899388365419035</v>
+        <v>0.7451931887554745</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-12 21:00:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Denver Nuggets</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>San Antonio Spurs</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.7607873703556378</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-12 21:30:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Boston Celtics</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Oklahoma City Thunder</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5903554062227555</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-12 22:30:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Chicago Bulls</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Los Angeles Lakers</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.6994576092751355</v>
       </c>
     </row>
   </sheetData>
@@ -605,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,330 +718,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Brooklyn Nets</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Brooklyn Nets</t>
+          <t>Houston Rockets</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.5338900739835579</v>
+        <v>0.4626488861327057</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Detroit Pistons</t>
+          <t>Denver Nuggets</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Sacramento Kings</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Toronto Raptors</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.4827779753068177</v>
+        <v>0.436097296384334</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Houston Rockets</t>
+          <t>Charlotte Hornets</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Milwaukee Bucks</t>
+          <t>Utah Jazz</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.3005046064918108</v>
+        <v>0.485288044971443</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Phoenix Suns</t>
+          <t>New York Knicks</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Boston Celtics</t>
+          <t>Toronto Raptors</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.627926628481095</v>
+        <v>0.558987577832024</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>San Antonio Spurs</t>
+          <t>New Orleans Pelicans</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minnesota Timberwolves</t>
+          <t>Cleveland Cavaliers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.6806914130463642</v>
+        <v>0.7107163444746127</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Los Angeles Lakers</t>
+          <t>Orlando Magic</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-03-10 00:00:00</t>
+          <t>2026-03-11 00:00:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Philadelphia 76ers</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies</t>
+          <t>Minnesota Timberwolves</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Memphis Grizzlies</t>
+          <t>LA Clippers</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.4006859410308615</v>
+        <v>0.6986770289848878</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Philadelphia 76ers</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Portland Trail Blazers</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0.3988693843428268</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Charlotte Hornets</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Sacramento Kings</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Indiana Pacers</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Sacramento Kings</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0.6955559714400453</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Sacramento Kings</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Miami Heat</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Washington Wizards</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Miami Heat</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>0.8107714131008203</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Miami Heat</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Golden State Warriors</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Chicago Bulls</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Chicago Bulls</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>0.4599169826326945</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Chicago Bulls</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-03-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Dallas Mavericks</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>0.8982030502084318</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Atlanta Hawks</t>
+          <t>LA Clippers</t>
         </is>
       </c>
     </row>

</xml_diff>